<commit_message>
Adiciona ponto de equilíbrio (break-even) com custos reais do Anti-Ruído
Nova aba "Custos (Ponto de Equilíbrio)" com preço de venda, custo
unitário e custo fixo mensal reais informados (R$100 / R$30 / R$56,4mil),
calculando margem de contribuição, ponto de equilíbrio em unidades/mês,
R$/mês e unidades/ano, além de uma simulação de lucro por volume de
vendas. Tamanho de mercado atualizado para 5 milhões (valor pesquisado)
e usado como fonte única também no cálculo de Market Share da aba
Métricas.
</commit_message>
<xml_diff>
--- a/docs/planilha-metricas-startup.xlsx
+++ b/docs/planilha-metricas-startup.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Dados" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Métricas" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Pontos de Virada" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Custos (Ponto de Equilíbrio)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -87,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,6 +103,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -191,6 +196,21 @@
     <comment ref="K7" authorId="0" shapeId="0">
       <text>
         <t>K-Factor = Clientes por Indicação ÷ Usuários Ativos (equivalente a (Convites por usuário) × (Taxa de conversão do convite) = (L/K)×(M/L) = M/K).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Nota</author>
+  </authors>
+  <commentList>
+    <comment ref="A19" authorId="0" shapeId="0">
+      <text>
+        <t>Ponto de equilíbrio calculado (arredondado para cima) — linha de referência.</t>
       </text>
     </comment>
   </commentList>
@@ -1180,7 +1200,7 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>10000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="3">
@@ -2529,4 +2549,384 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Parâmetros de custo (produto físico — compra única, sem recorrência)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Preço de Venda (R$)</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Custo Unitário / COGS (R$)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Custo Fixo Mensal (R$)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>56400</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tamanho do Mercado (clientes potenciais)</t>
+        </is>
+      </c>
+      <c r="B5" s="11">
+        <f>Métricas!B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Cálculos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Margem de Contribuição Unitária (R$)</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>B2-B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Margem de Contribuição (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>B8/B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio (unidades/mês)</t>
+        </is>
+      </c>
+      <c r="B10" s="12">
+        <f>B4/B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio (R$/mês)</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>B10*B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio (unidades/ano)</t>
+        </is>
+      </c>
+      <c r="B12" s="12">
+        <f>B10*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>% do mercado necessário para break-even (1 mês)</t>
+        </is>
+      </c>
+      <c r="B13" s="13">
+        <f>B10/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Simulação de volume de vendas (unidades/mês)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Unidades/mês</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Receita (R$)</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Custo Variável (R$)</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Custo Fixo (R$)</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Lucro/Prejuízo Mensal (R$)</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>% do Mercado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B17" s="3">
+        <f>A17*$B$2</f>
+        <v/>
+      </c>
+      <c r="C17" s="3">
+        <f>A17*$B$3</f>
+        <v/>
+      </c>
+      <c r="D17" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E17" s="3">
+        <f>B17-C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="13">
+        <f>A17/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B18" s="3">
+        <f>A18*$B$2</f>
+        <v/>
+      </c>
+      <c r="C18" s="3">
+        <f>A18*$B$3</f>
+        <v/>
+      </c>
+      <c r="D18" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E18" s="3">
+        <f>B18-C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="13">
+        <f>A18/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <f>ROUNDUP(B10,0)</f>
+        <v/>
+      </c>
+      <c r="B19" s="3">
+        <f>A19*$B$2</f>
+        <v/>
+      </c>
+      <c r="C19" s="3">
+        <f>A19*$B$3</f>
+        <v/>
+      </c>
+      <c r="D19" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E19" s="3">
+        <f>B19-C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>A19/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B20" s="3">
+        <f>A20*$B$2</f>
+        <v/>
+      </c>
+      <c r="C20" s="3">
+        <f>A20*$B$3</f>
+        <v/>
+      </c>
+      <c r="D20" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E20" s="3">
+        <f>B20-C20-D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="13">
+        <f>A20/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B21" s="3">
+        <f>A21*$B$2</f>
+        <v/>
+      </c>
+      <c r="C21" s="3">
+        <f>A21*$B$3</f>
+        <v/>
+      </c>
+      <c r="D21" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E21" s="3">
+        <f>B21-C21-D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="13">
+        <f>A21/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B22" s="3">
+        <f>A22*$B$2</f>
+        <v/>
+      </c>
+      <c r="C22" s="3">
+        <f>A22*$B$3</f>
+        <v/>
+      </c>
+      <c r="D22" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E22" s="3">
+        <f>B22-C22-D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="13">
+        <f>A22/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B23" s="3">
+        <f>A23*$B$2</f>
+        <v/>
+      </c>
+      <c r="C23" s="3">
+        <f>A23*$B$3</f>
+        <v/>
+      </c>
+      <c r="D23" s="3">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="E23" s="3">
+        <f>B23-C23-D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="13">
+        <f>A23/$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Como usar: preencha B2:B4 (preço, custo unitário e custo fixo mensal) com os números reais — o Ponto de Equilíbrio e a simulação abaixo recalculam sozinhos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>O Tamanho do Mercado (B5) vem da mesma célula usada na aba Métricas (Market Share) — mude em um lugar só.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Este produto é de compra única (hardware), então aqui não se aplica churn/LTV/MRR — o equivalente de 'ponto de equilíbrio' de um negócio recorrente é vender, todo mês, unidades suficientes para cobrir o custo fixo do mês.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>